<commit_message>
Surya Update new feature file
</commit_message>
<xml_diff>
--- a/src/main/resources/Surya_Program_Field_Values.xlsx
+++ b/src/main/resources/Surya_Program_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stealth User1\Desktop\Dev_Home\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ACDC49C-57F5-4BE4-B8B8-B348CE4F15F5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A1DBC2-60C1-4FA8-9142-9AB5D2DA0B5B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{5C4D9AE9-7F6A-4097-8B3C-560C6A890586}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" activeTab="1" xr2:uid="{5C4D9AE9-7F6A-4097-8B3C-560C6A890586}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -87,16 +87,16 @@
     <t>Department of Education</t>
   </si>
   <si>
-    <t>Program for Newborn Screening</t>
-  </si>
-  <si>
-    <t>PGNS</t>
-  </si>
-  <si>
-    <t>Surya automation Data</t>
+    <t>Youth Program</t>
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>PGYH</t>
+  </si>
+  <si>
+    <t>Automation Data Feb 4</t>
   </si>
 </sst>
 </file>
@@ -536,7 +536,7 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -547,7 +547,7 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -587,7 +587,7 @@
         <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -609,7 +609,7 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>